<commit_message>
data: daily quota update 2026-07-06
</commit_message>
<xml_diff>
--- a/data/published/Quota_History.xlsx
+++ b/data/published/Quota_History.xlsx
@@ -6826,23 +6826,23 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>0</v>
+        <v>103743.08</v>
       </c>
       <c r="G136" t="n">
-        <v>0</v>
+        <v>20219.69</v>
       </c>
       <c r="H136" t="n">
-        <v>0</v>
+        <v>19.49</v>
       </c>
       <c r="I136" t="n">
-        <v>0</v>
+        <v>83523.39999999999</v>
       </c>
       <c r="J136" t="n">
-        <v>0</v>
+        <v>80.51000000000001</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
-          <t>failed</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -10868,19 +10868,19 @@
         </is>
       </c>
       <c r="F222" t="n">
-        <v>0</v>
+        <v>896.35</v>
       </c>
       <c r="G222" t="n">
-        <v>0</v>
+        <v>284.79</v>
       </c>
       <c r="H222" t="n">
-        <v>0</v>
+        <v>31.77</v>
       </c>
       <c r="I222" t="n">
-        <v>0</v>
+        <v>611.5599999999999</v>
       </c>
       <c r="J222" t="n">
-        <v>0</v>
+        <v>68.23</v>
       </c>
       <c r="K222" t="inlineStr">
         <is>

</xml_diff>